<commit_message>
Fix sample Excel file to match exact Danalog column structure
- Updated sample file with all 24 columns from original Danalog catalog
- Exact column names: ש.לפריט, דאנאקוד, שם, ק.מחלקה, ת.מחלקה, etc.
- 10 realistic book entries with proper Hebrew text
- Matches structure of Danalog_0-1070616.xlsx for seamless testing

Co-Authored-By: Claude Sonnet 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/דוגמה_קטלוג_להעלאה.xlsx
+++ b/דוגמה_קטלוג_להעלאה.xlsx
@@ -425,450 +425,810 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:X11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>ש.לפריט</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
           <t>דאנאקוד</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>שם</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>ק.מחלקה</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>ת.מחלקה</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>מחיר</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>מ.מיוחד</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>מ.מיוחד1</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>לימוד</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>מאושר</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>ק.יצרן</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>יצרן</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>ק.מחבר</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>מחבר</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>ת.מחלקה</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>מחיר</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>ק.נושא</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>נושא</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>אזל</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>ברקוד</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>ברקוד-נ</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>פמי.ר</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>פמי.מ</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>ת.פתיחה</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>נושא</t>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>ת.עדכון</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>ת.מה.ראשונה</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>101-10001</t>
-        </is>
+      <c r="A2" t="n">
+        <v>1</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>הארי פוטר ואבן החכמים</t>
+          <t>101-10541</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>ג.ק. רולינג</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>ספרות ילדים</t>
-        </is>
-      </c>
-      <c r="E2" t="n">
-        <v>45.9</v>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>9780747532699</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
+          <t>שלום לך קליפורניה/אליסטר מקלין *יחולי*</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>101</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>קריאה</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>29.9</v>
+      </c>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>מקלין אליסטר</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>מקלין אליסטר</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>ספרות - מתורגמת</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr"/>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>010100105413</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr"/>
+      <c r="T2" t="inlineStr"/>
+      <c r="U2" t="inlineStr"/>
+      <c r="V2" t="inlineStr">
         <is>
           <t>2024-01-15</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>פנטזיה</t>
-        </is>
-      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>2024-01-15</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>101-10002</t>
-        </is>
+      <c r="A3" t="n">
+        <v>2</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>שלום לך בסלון</t>
+          <t>101-10612</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>מאיר שלו</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>ספרות מתורגמת</t>
-        </is>
-      </c>
-      <c r="E3" t="n">
-        <v>39.9</v>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>9789650123456</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
+          <t>שלום לך סיינוגיע/נידה נינה *יחולי* (אזן)</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>101</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>קריאה</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>25</v>
+      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>נידה נינה</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>נידה נינה</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>ספרות - מתורגמת</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr"/>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>010100106120</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr"/>
+      <c r="T3" t="inlineStr"/>
+      <c r="U3" t="inlineStr"/>
+      <c r="V3" t="inlineStr">
         <is>
           <t>2024-02-20</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>רומן</t>
-        </is>
-      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>2024-02-20</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>101-10003</t>
-        </is>
+      <c r="A4" t="n">
+        <v>3</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>עליזה וחבריה</t>
+          <t>101-40324</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>גלילה רון-פדר-עמית</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
+          <t>דנדיו ודנדין שמרי השלום/שרה *יחולי*</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>101</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>קריאה</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>29</v>
+      </c>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>שרד אזן</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>שרד אזן</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr">
         <is>
           <t>ספרות ילדים</t>
         </is>
       </c>
-      <c r="E4" t="n">
-        <v>29.9</v>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>9789653561234</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
+      <c r="Q4" t="inlineStr"/>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>010100403243</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr"/>
+      <c r="T4" t="inlineStr"/>
+      <c r="U4" t="inlineStr"/>
+      <c r="V4" t="inlineStr">
         <is>
           <t>2024-03-10</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>ילדים</t>
-        </is>
-      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>2024-03-10</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>101-10004</t>
-        </is>
+      <c r="A5" t="n">
+        <v>4</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>מסע אל העבר</t>
+          <t>10-272708</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>עמוס עוז</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>ספרות עברית</t>
-        </is>
-      </c>
-      <c r="E5" t="n">
-        <v>55</v>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>9789650234567</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
+          <t>הרי שלום והודה על הנהים/דאנלבס אדמס</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>10</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>תרגום</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>89</v>
+      </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>אדמס דאנלבס</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>אדמס דאנלבס</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>סיפור - מקור</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr"/>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>001002727087</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr"/>
+      <c r="T5" t="inlineStr"/>
+      <c r="U5" t="inlineStr"/>
+      <c r="V5" t="inlineStr">
         <is>
           <t>2024-01-05</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>רומן</t>
-        </is>
-      </c>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>2024-01-05</t>
+        </is>
+      </c>
+      <c r="X5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>101-10005</t>
-        </is>
+      <c r="A6" t="n">
+        <v>5</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>סיפורי ילדים</t>
+          <t>10-275646</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>לאה גולדברג</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>שירה</t>
-        </is>
-      </c>
-      <c r="E6" t="n">
-        <v>25</v>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>9789650345678</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
+          <t>אל נא תאמר לי שלום/יוסי ונקסון יוסי</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>10</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>תרגום</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>30</v>
+      </c>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>ונקסון יוסי</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>ונקסון יוסי</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>סיפור - מקור</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr"/>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>001002756469</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr"/>
+      <c r="T6" t="inlineStr"/>
+      <c r="U6" t="inlineStr"/>
+      <c r="V6" t="inlineStr">
         <is>
           <t>2024-04-12</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>שירה</t>
-        </is>
-      </c>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>2024-04-12</t>
+        </is>
+      </c>
+      <c r="X6" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>102-20001</t>
-        </is>
+      <c r="A7" t="n">
+        <v>6</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>המדריך לגינון</t>
+          <t>10-277366</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>דוד כהן</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>גינון</t>
-        </is>
-      </c>
-      <c r="E7" t="n">
-        <v>35</v>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>9789650456789</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
+          <t>טבח התווכל/שלום עליכם</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>10</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>מקור</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>89</v>
+      </c>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>שלום עליכם</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>שלום עליכם</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>מקור</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr"/>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>001002773660</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr"/>
+      <c r="T7" t="inlineStr"/>
+      <c r="U7" t="inlineStr"/>
+      <c r="V7" t="inlineStr">
         <is>
           <t>2024-05-18</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>גינון ונוי</t>
-        </is>
-      </c>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>2024-05-18</t>
+        </is>
+      </c>
+      <c r="X7" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>102-20002</t>
-        </is>
+      <c r="A8" t="n">
+        <v>7</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>בישול בריא</t>
+          <t>10-277493</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>רחל לוי</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>בישול</t>
-        </is>
-      </c>
-      <c r="E8" t="n">
-        <v>42</v>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>9789650567890</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
+          <t>סיפורי תווה/שלום עליכם</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>10</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>מקור</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>98</v>
+      </c>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>שלום עליכם</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>שלום עליכם</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr"/>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>מקור</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr"/>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>001002774930</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr"/>
+      <c r="T8" t="inlineStr"/>
+      <c r="U8" t="inlineStr"/>
+      <c r="V8" t="inlineStr">
         <is>
           <t>2024-06-22</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>מתכונים</t>
-        </is>
-      </c>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>2024-06-22</t>
+        </is>
+      </c>
+      <c r="X8" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>103-30001</t>
-        </is>
+      <c r="A9" t="n">
+        <v>8</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>ההיסטוריה של ישראל</t>
+          <t>10-277914</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>יעקב שביט</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>היסטוריה</t>
-        </is>
-      </c>
-      <c r="E9" t="n">
-        <v>68</v>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>9789650678901</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
+          <t>הרי שלום והודה על הנהים/מחדוד/דאנלבס אדמס</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>10</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>תרגום</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>92</v>
+      </c>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>אדמס דאנלבס</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>אדמס דאנלבס</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr"/>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>סיפור מחודד/ד.אדמס</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr"/>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>001002779140</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr"/>
+      <c r="T9" t="inlineStr"/>
+      <c r="U9" t="inlineStr"/>
+      <c r="V9" t="inlineStr">
         <is>
           <t>2024-07-08</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>מדינת ישראל</t>
-        </is>
-      </c>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>2024-07-08</t>
+        </is>
+      </c>
+      <c r="X9" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>103-30002</t>
-        </is>
+      <c r="A10" t="n">
+        <v>9</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>ספר מתמטיקה לכיתה ז</t>
+          <t>10-279149</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>משרד החינוך</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>לימוד</t>
-        </is>
-      </c>
-      <c r="E10" t="n">
-        <v>45</v>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>9789650789012</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
+          <t>שלום לקנאים: שלום מחשבות/עמוס עזו</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>10</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>קריאה</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>39.9</v>
+      </c>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>עמוס עזו</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>עמוס עזו</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr"/>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>שלום</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr"/>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>001002791490</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr"/>
+      <c r="T10" t="inlineStr"/>
+      <c r="U10" t="inlineStr"/>
+      <c r="V10" t="inlineStr">
         <is>
           <t>2024-08-14</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>מתמטיקה</t>
-        </is>
-      </c>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>2024-08-14</t>
+        </is>
+      </c>
+      <c r="X10" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>104-40001</t>
-        </is>
+      <c r="A11" t="n">
+        <v>10</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>אנגלית למתחילים</t>
+          <t>103-112</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>ג'ון סמית</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>לימוד</t>
-        </is>
-      </c>
-      <c r="E11" t="n">
-        <v>38</v>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>9789650890123</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
+          <t>אופסי המנוח: יבר לו של שלום/חנה ודינמן</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>103</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>קריאה</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>35</v>
+      </c>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>ודינמן חנה</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>ודינמן חנה</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr"/>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>אופסי</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr"/>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>00100271087</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr"/>
+      <c r="T11" t="inlineStr"/>
+      <c r="U11" t="inlineStr"/>
+      <c r="V11" t="inlineStr">
         <is>
           <t>2024-09-03</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>שפה אנגלית</t>
-        </is>
-      </c>
+      <c r="W11" t="inlineStr">
+        <is>
+          <t>2024-09-03</t>
+        </is>
+      </c>
+      <c r="X11" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>